<commit_message>
clean up prediction results and editted readme
</commit_message>
<xml_diff>
--- a/nba_prediction_log.xlsx
+++ b/nba_prediction_log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tjwill/TJ's Stuff/Portfolio/nba_predictor/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CA1A72CA-E1D3-A142-A4F0-0FB51EE684FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{539B6DF2-5E12-0348-AF21-B8EE43AB6AF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="33">
   <si>
     <t>NBA FINALS 2026 — SENTIMENT MODEL PREDICTION LOG</t>
   </si>
@@ -92,9 +92,6 @@
     <t>Finals G5</t>
   </si>
   <si>
-    <t>TBD</t>
-  </si>
-  <si>
     <t>Finals G6</t>
   </si>
   <si>
@@ -113,9 +110,6 @@
     <t>Games Predicted</t>
   </si>
   <si>
-    <t>1. Fill in Home &amp; Away Sentiment from sentiment.py output</t>
-  </si>
-  <si>
     <t>Correct</t>
   </si>
   <si>
@@ -132,14 +126,21 @@
   </si>
   <si>
     <t>5. Re-run full pipeline before next game, update next row</t>
+  </si>
+  <si>
+    <t>✗</t>
+  </si>
+  <si>
+    <t>1. Fill in Home &amp; Away Sentiment from predict.py output</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
@@ -236,14 +237,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF533483"/>
-        <bgColor rgb="FF533483"/>
+        <fgColor rgb="FF1A1A2E"/>
+        <bgColor rgb="FF1A1A2E"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1A1A2E"/>
-        <bgColor rgb="FF1A1A2E"/>
+        <fgColor theme="3" tint="-0.249977111117893"/>
+        <bgColor rgb="FF533483"/>
       </patternFill>
     </fill>
   </fills>
@@ -274,7 +275,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -282,9 +283,6 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -295,30 +293,42 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -638,34 +648,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="15"/>
-      <c r="I1" s="15"/>
-      <c r="J1" s="15"/>
-      <c r="K1" s="15"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
     </row>
     <row r="2" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
-      <c r="J2" s="15"/>
-      <c r="K2" s="15"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="16"/>
+      <c r="K2" s="16"/>
     </row>
     <row r="4" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
@@ -706,7 +716,7 @@
       <c r="A5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="11" t="s">
         <v>14</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -715,47 +725,55 @@
       <c r="D5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="17">
-        <v>0.57142857142857095</v>
-      </c>
-      <c r="H5" s="3" t="s">
+      <c r="E5" s="2">
+        <v>0.2238</v>
+      </c>
+      <c r="F5" s="2">
+        <v>0.22559999999999999</v>
+      </c>
+      <c r="G5" s="2">
+        <v>-1.8E-3</v>
+      </c>
+      <c r="H5" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-      <c r="K5" s="4" t="s">
+      <c r="I5" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K5" s="3" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6" s="5" t="s">
+      <c r="B6" s="10">
+        <v>46186</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="5"/>
-      <c r="K6" s="6"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="4"/>
+      <c r="H6" s="20"/>
+      <c r="I6" s="20"/>
+      <c r="J6" s="4"/>
+      <c r="K6" s="5"/>
     </row>
     <row r="7" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" s="2" t="s">
         <v>19</v>
+      </c>
+      <c r="B7" s="10">
+        <v>46189</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>15</v>
@@ -766,136 +784,136 @@
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
+      <c r="H7" s="19"/>
+      <c r="I7" s="19"/>
       <c r="J7" s="2"/>
-      <c r="K7" s="4" t="s">
+      <c r="K7" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="4" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="5" t="s">
+      <c r="B8" s="10">
+        <v>46192</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
+      <c r="G8" s="4"/>
+      <c r="H8" s="20"/>
+      <c r="I8" s="20"/>
+      <c r="J8" s="4"/>
+      <c r="K8" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A10" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="B8" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5"/>
-      <c r="J8" s="5"/>
-      <c r="K8" s="6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A10" s="11" t="s">
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="E10" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="12"/>
-      <c r="C10" s="12"/>
-      <c r="E10" s="11" t="s">
+      <c r="F10" s="13"/>
+      <c r="G10" s="13"/>
+      <c r="H10" s="13"/>
+      <c r="I10" s="13"/>
+      <c r="J10" s="13"/>
+      <c r="K10" s="13"/>
+    </row>
+    <row r="11" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="F10" s="12"/>
-      <c r="G10" s="12"/>
-      <c r="H10" s="12"/>
-      <c r="I10" s="12"/>
-      <c r="J10" s="12"/>
-      <c r="K10" s="12"/>
-    </row>
-    <row r="11" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="B11" s="9">
+      <c r="B11" s="8">
         <f>COUNTA(H5:H8)</f>
         <v>1</v>
       </c>
-      <c r="C11" s="12"/>
-      <c r="E11" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="F11" s="12"/>
-      <c r="G11" s="12"/>
-      <c r="H11" s="12"/>
-      <c r="I11" s="12"/>
-      <c r="J11" s="12"/>
-      <c r="K11" s="12"/>
+      <c r="C11" s="13"/>
+      <c r="E11" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="F11" s="13"/>
+      <c r="G11" s="13"/>
+      <c r="H11" s="13"/>
+      <c r="I11" s="13"/>
+      <c r="J11" s="13"/>
+      <c r="K11" s="13"/>
     </row>
     <row r="12" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" s="9">
+      <c r="A12" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="8">
         <f>COUNTIF(J5:J8,"✓")</f>
         <v>0</v>
       </c>
-      <c r="C12" s="12"/>
-      <c r="E12" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="F12" s="12"/>
-      <c r="G12" s="12"/>
-      <c r="H12" s="12"/>
-      <c r="I12" s="12"/>
-      <c r="J12" s="12"/>
-      <c r="K12" s="12"/>
+      <c r="C12" s="13"/>
+      <c r="E12" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="F12" s="13"/>
+      <c r="G12" s="13"/>
+      <c r="H12" s="13"/>
+      <c r="I12" s="13"/>
+      <c r="J12" s="13"/>
+      <c r="K12" s="13"/>
     </row>
     <row r="13" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="B13" s="10">
+      <c r="A13" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" s="9">
         <f>IFERROR(B12/B11,0)</f>
         <v>0</v>
       </c>
-      <c r="C13" s="12"/>
-      <c r="E13" s="13" t="s">
+      <c r="C13" s="13"/>
+      <c r="E13" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="F13" s="13"/>
+      <c r="G13" s="13"/>
+      <c r="H13" s="13"/>
+      <c r="I13" s="13"/>
+      <c r="J13" s="13"/>
+      <c r="K13" s="13"/>
+    </row>
+    <row r="14" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="6"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6"/>
+      <c r="E14" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="F14" s="13"/>
+      <c r="G14" s="13"/>
+      <c r="H14" s="13"/>
+      <c r="I14" s="13"/>
+      <c r="J14" s="13"/>
+      <c r="K14" s="13"/>
+    </row>
+    <row r="15" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="6"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="E15" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="F13" s="12"/>
-      <c r="G13" s="12"/>
-      <c r="H13" s="12"/>
-      <c r="I13" s="12"/>
-      <c r="J13" s="12"/>
-      <c r="K13" s="12"/>
-    </row>
-    <row r="14" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="7"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="E14" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="F14" s="12"/>
-      <c r="G14" s="12"/>
-      <c r="H14" s="12"/>
-      <c r="I14" s="12"/>
-      <c r="J14" s="12"/>
-      <c r="K14" s="12"/>
-    </row>
-    <row r="15" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="7"/>
-      <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
-      <c r="E15" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="F15" s="12"/>
-      <c r="G15" s="12"/>
-      <c r="H15" s="12"/>
-      <c r="I15" s="12"/>
-      <c r="J15" s="12"/>
-      <c r="K15" s="12"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="13"/>
+      <c r="H15" s="13"/>
+      <c r="I15" s="13"/>
+      <c r="J15" s="13"/>
+      <c r="K15" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>